<commit_message>
Checked for final review
</commit_message>
<xml_diff>
--- a/Energy community potential model/_assumptions.xlsx
+++ b/Energy community potential model/_assumptions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\s124129\Documents\GitHub\Energy-community-potential-model\Energy community potential model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naudl\Documents\GitHub\Energy-community-potential-model\Energy community potential model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E1E6A4A-D38B-44BB-BF21-EC70D6897FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A74585-D2BD-4AD5-95CD-2A316586F2FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="3" xr2:uid="{7889CB36-7083-4D16-B0FE-16DC7F037511}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{7889CB36-7083-4D16-B0FE-16DC7F037511}"/>
   </bookViews>
   <sheets>
     <sheet name="global_assumptions" sheetId="6" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="110">
   <si>
     <t>Parameter</t>
   </si>
@@ -395,18 +395,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -425,7 +419,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -761,12 +755,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B0C4BD5-7A03-4979-9B24-44A967EC7A8F}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.140625" customWidth="1"/>
+    <col min="1" max="1" width="32.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>73</v>
       </c>
@@ -774,7 +768,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>65</v>
       </c>
@@ -782,7 +776,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>66</v>
       </c>
@@ -790,7 +784,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>67</v>
       </c>
@@ -798,7 +792,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>68</v>
       </c>
@@ -806,7 +800,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>70</v>
       </c>
@@ -814,7 +808,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>69</v>
       </c>
@@ -822,7 +816,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>72</v>
       </c>
@@ -830,7 +824,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -846,12 +840,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2C6F96C-7FCC-4470-983E-20F0B68A4987}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="1" max="1" width="23.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>93</v>
       </c>
@@ -871,7 +865,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -893,7 +887,7 @@
         <v>0.19600000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -918,7 +912,7 @@
         <v>0.19725909494232474</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -943,7 +937,7 @@
         <v>0.25393077301821765</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>87</v>
       </c>
@@ -967,7 +961,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>82</v>
       </c>
@@ -991,7 +985,7 @@
         <v>0.24285714285714285</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>85</v>
       </c>
@@ -1015,7 +1009,7 @@
         <v>0.22714285714285715</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>86</v>
       </c>
@@ -1023,7 +1017,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -1039,14 +1033,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16EDA63B-8F45-4FF0-9A5F-7ED4FA8CF17E}">
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>80</v>
       </c>
@@ -1063,7 +1057,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -1082,7 +1076,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -1101,7 +1095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -1120,7 +1114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>87</v>
       </c>
@@ -1134,7 +1128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -1153,7 +1147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1172,7 +1166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -1191,7 +1185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -1210,7 +1204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>82</v>
       </c>
@@ -1224,7 +1218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -1242,7 +1236,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -1257,7 +1251,7 @@
         <v>0.82918739635157546</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>85</v>
       </c>
@@ -1271,7 +1265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>86</v>
       </c>
@@ -1285,7 +1279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>107</v>
       </c>
@@ -1300,7 +1294,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>107</v>
       </c>
@@ -1315,7 +1309,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>75</v>
       </c>
@@ -1334,7 +1328,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>75</v>
       </c>
@@ -1353,7 +1347,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>75</v>
       </c>
@@ -1372,7 +1366,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>75</v>
       </c>
@@ -1391,7 +1385,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>95</v>
       </c>
@@ -1406,7 +1400,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -1421,7 +1415,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -1440,7 +1434,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1459,7 +1453,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -1478,7 +1472,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1500,13 +1494,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D89132D8-0BA9-4425-B509-CC7F5584808F}">
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" customWidth="1"/>
+    <col min="1" max="1" width="21.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>28</v>
       </c>
@@ -1525,11 +1519,8 @@
       <c r="G1" t="s">
         <v>85</v>
       </c>
-      <c r="H1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -1537,7 +1528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -1548,7 +1539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -1562,7 +1553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>87</v>
       </c>
@@ -1579,7 +1570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>82</v>
       </c>
@@ -1595,11 +1586,11 @@
       <c r="E6" s="3">
         <v>0.4</v>
       </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>85</v>
       </c>
@@ -1619,23 +1610,6 @@
         <v>0.4</v>
       </c>
       <c r="G7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>0.5</v>
-      </c>
-      <c r="D8">
-        <v>0.5</v>
-      </c>
-      <c r="E8">
-        <v>0.4</v>
-      </c>
-      <c r="H8">
         <v>1</v>
       </c>
     </row>
@@ -1647,12 +1621,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2366E1BF-C2F7-4663-8D71-BD7975399B57}">
   <dimension ref="A1:J18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="1" max="1" width="27.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1681,7 +1655,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -1707,7 +1681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1741,7 +1715,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1775,7 +1749,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>60</v>
       </c>
@@ -1809,7 +1783,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1843,7 +1817,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -1872,7 +1846,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -1898,7 +1872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -1924,7 +1898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1952,7 +1926,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -1981,7 +1955,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -2007,7 +1981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -2033,7 +2007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -2067,7 +2041,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -2101,7 +2075,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -2135,7 +2109,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -2163,7 +2137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -2197,16 +2171,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C237FD6B-E6B1-4A3E-AEC6-1B0A088B4EBA}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" customWidth="1"/>
+    <col min="1" max="1" width="5.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="107.28515625" customWidth="1"/>
+    <col min="5" max="5" width="107.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2226,7 +2200,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2246,7 +2220,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2266,7 +2240,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2286,7 +2260,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2306,7 +2280,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2334,12 +2308,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F64D8631-75B4-44F4-A1D9-F89D31ED0FA6}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>58</v>
       </c>
@@ -2350,7 +2324,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -2362,7 +2336,7 @@
         <v>0.496</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>29</v>
       </c>
@@ -2376,7 +2350,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>31</v>
       </c>
@@ -2390,7 +2364,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>32</v>
       </c>
@@ -2404,7 +2378,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -2418,7 +2392,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>36</v>
       </c>
@@ -2432,7 +2406,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -2446,7 +2420,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -2460,7 +2434,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -2474,7 +2448,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -2488,7 +2462,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>41</v>
       </c>
@@ -2502,7 +2476,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -2516,7 +2490,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -2530,7 +2504,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -2544,7 +2518,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -2558,7 +2532,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>46</v>
       </c>
@@ -2572,7 +2546,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -2587,7 +2561,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>57</v>
       </c>

</xml_diff>